<commit_message>
Revert Excel null display to blank cells, give date/numeric columns real Excel types, wipe test-run logs
- build_excel.py: drop the "미기재" string fill — null stays a real blank cell so date/number
  columns keep proper Excel types instead of being coerced to text
- release_date/last_modified_date cast to datetime (date_format="YYYY-MM-DD"); parameters/
  context_length cast to numeric with integer display format
- clear logs/ (ai_outputs.json, last_run_changes.json, last_run_excluded.json,
  pending_ai_inputs.json) — these are per-run scratch, regenerated by the next pipeline run

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/huggingface_models_2026-07-19.xlsx
+++ b/output/huggingface_models_2026-07-19.xlsx
@@ -17,7 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -56,11 +59,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -634,20 +639,16 @@
           <t>기타(hyperclovax)</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2025-12-23</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-07-14</t>
-        </is>
-      </c>
-      <c r="M2" t="n">
+      <c r="K2" s="2" t="n">
+        <v>46014</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="M2" s="3" t="n">
         <v>33313410304</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" s="3" t="n">
         <v>131072</v>
       </c>
       <c r="O2" t="inlineStr">
@@ -665,41 +666,13 @@
           <t>베이스 모델</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr">
         <is>
           <t>2025-05</t>
@@ -757,20 +730,16 @@
           <t>기타(hyperclovax-seed)</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>2025-07-21</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
+      <c r="K3" s="2" t="n">
+        <v>45859</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>46170</v>
+      </c>
+      <c r="M3" s="3" t="n">
         <v>14748112896</v>
       </c>
-      <c r="N3" t="n">
+      <c r="N3" s="3" t="n">
         <v>32768</v>
       </c>
       <c r="O3" t="inlineStr">
@@ -788,11 +757,7 @@
           <t>경량화·증류 모델</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
           <t>MMLU=71.21;BigBench-Hard=62.16;Hellaswag=61.25;Winogrande=75.93;PIQA=77.91;ARC-challenge=62.46;SocialIQa=52.05;MT-Bench=8.8313;Arena-Hard-v0.1=58.26;GPT4Eval=82.00;CLIcK=72.08;HAERAE-Bench=85.06;KOBEST=85.70;KorMedMCQA=64.11;KMMLU=54.28;KoBigBench=74.82;KoCommonGEN-v2=66.82;CSAT-ko-2025=75.16;KoBALT=45.00;LogicKor=8.74</t>
@@ -803,31 +768,15 @@
           <t>GSM8k=95.53;MATH500=93.80;HumanEval=94.51;MBPP=87.59</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr">
         <is>
           <t>CLIcK=72.08;HAERAE-Bench=85.06;KOBEST=85.70;KorMedMCQA=64.11;KMMLU=54.28;KoBigBench=74.82;KoCommonGEN-v2=66.82;CSAT-ko-2025=75.16;KoBALT=45.00;LogicKor=8.74</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -880,20 +829,16 @@
           <t>기타(hyperclovax)</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>2025-12-23</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>2026-01-06</t>
-        </is>
-      </c>
-      <c r="M4" t="n">
+      <c r="K4" s="2" t="n">
+        <v>46014</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>46028</v>
+      </c>
+      <c r="M4" s="3" t="n">
         <v>10741664520</v>
       </c>
-      <c r="N4" t="n">
+      <c r="N4" s="3" t="n">
         <v>32768</v>
       </c>
       <c r="O4" t="inlineStr">
@@ -911,41 +856,13 @@
           <t>베이스 모델</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr">
         <is>
           <t>2025-05</t>
@@ -973,11 +890,7 @@
           <t>https://huggingface.co/naver-hyperclovax/HyperCLOVAX-SEED-Vision-Instruct-3B</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>적은 비전 토큰으로도 한국어 VQA·이미지해석에서 동급 오픈소스 모델 대비 우수한 경량 VLM</t>
@@ -1003,20 +916,16 @@
           <t>기타(hyperclovax-seed)</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>2025-04-22</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>2025-09-16</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
+      <c r="K5" s="2" t="n">
+        <v>45769</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>45916</v>
+      </c>
+      <c r="M5" s="3" t="n">
         <v>3721243520</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" s="3" t="n">
         <v>16384</v>
       </c>
       <c r="O5" t="inlineStr">
@@ -1044,31 +953,19 @@
           <t>KMMLU=44.22;HAE-RAE=64.99;CLiCK=55.99;KoBEST=71.80</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr">
         <is>
           <t>VideoMME=48.2;NAVER-TV-CLIP=61.0;VideoChatGPT=53.6;PerceptionTest=55.2;ActivityNet-QA=50.6;KoNet=69.2;MMBench-Val=81.8;TextVQA-Val=79.2;Korean VisIT-Bench=37.0</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr">
         <is>
           <t>KMMLU=44.22;HAE-RAE=64.99;CLiCK=55.99;KoBEST=71.80;VideoMME=48.2;NAVER-TV-CLIP=61.0;VideoChatGPT=53.6;KoNet=69.2;Korean VisIT-Bench=37.0</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr">
         <is>
           <t>2024-08</t>
@@ -1096,11 +993,7 @@
           <t>https://huggingface.co/naver-hyperclovax/HyperCLOVAX-SEED-Text-Instruct-0.5B</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>동급 대비 수학·한국어 성능 우수, 학습비용 39배 절감돼 엣지 기기 배포에 적합한 소형 모델</t>
@@ -1126,20 +1019,16 @@
           <t>기타(hyperclovax-seed)</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>2025-04-22</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>2025-07-21</t>
-        </is>
-      </c>
-      <c r="M6" t="n">
+      <c r="K6" s="2" t="n">
+        <v>45769</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>45859</v>
+      </c>
+      <c r="M6" s="3" t="n">
         <v>566281216</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N6" s="3" t="n">
         <v>4096</v>
       </c>
       <c r="O6" t="inlineStr">
@@ -1167,31 +1056,15 @@
           <t>KMMLU=38.15;HAE-RAE=56.19;CLiCK=44.46;KoBEST=62.99</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr">
         <is>
           <t>KMMLU=38.15;HAE-RAE=56.19;CLiCK=44.46;KoBEST=62.99</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr">
         <is>
           <t>2025-01</t>
@@ -1219,11 +1092,7 @@
           <t>https://huggingface.co/Supertone/supertonic-3</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>5개에서 31개 언어로 확장하고 낭독 안정성을 개선한 99M 파라미터 온디바이스 TTS</t>
@@ -1249,29 +1118,17 @@
           <t>OpenRAIL</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
+      <c r="K7" s="2" t="n">
+        <v>46148</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>46160</v>
+      </c>
+      <c r="M7" s="3" t="n">
         <v>99000000</v>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="N7" s="3" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>Onnx</t>
@@ -1282,46 +1139,14 @@
           <t>베이스 모델</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1344,11 +1169,7 @@
           <t>https://huggingface.co/Supertone/supertonic-2</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>동일한 추론 속도를 유지하며 5개 언어로 확장된 66M 경량 온디바이스 TTS</t>
@@ -1374,29 +1195,17 @@
           <t>OpenRAIL</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>2026-01-06</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>2026-01-06</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
+      <c r="K8" s="2" t="n">
+        <v>46028</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>46028</v>
+      </c>
+      <c r="M8" s="3" t="n">
         <v>66000000</v>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="N8" s="3" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
           <t>Onnx</t>
@@ -1412,41 +1221,13 @@
           <t>Supertone/supertonic</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1469,11 +1250,7 @@
           <t>https://huggingface.co/Supertone/supertonic</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>M4 Pro CPU 기준 실시간 대비 최대 167배 빠른 66M 경량 온디바이스 TTS</t>
@@ -1499,29 +1276,17 @@
           <t>OpenRAIL</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>2025-11-18</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>2025-12-10</t>
-        </is>
-      </c>
-      <c r="M9" t="n">
+      <c r="K9" s="2" t="n">
+        <v>45979</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>46001</v>
+      </c>
+      <c r="M9" s="3" t="n">
         <v>66000000</v>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="N9" s="3" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
           <t>Onnx</t>
@@ -1532,46 +1297,14 @@
           <t>베이스 모델</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="X9" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1773,11 +1506,7 @@
           <t>https://huggingface.co/Supertone/supertonic</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>M4 Pro CPU 기준 실시간 대비 최대 167배 빠른 66M 경량 온디바이스 TTS</t>
@@ -1803,29 +1532,17 @@
           <t>OpenRAIL</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2025-11-18</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2025-12-10</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
+      <c r="L2" s="2" t="n">
+        <v>45979</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>46001</v>
+      </c>
+      <c r="N2" s="3" t="n">
         <v>66000000</v>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="O2" s="3" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
         <is>
           <t>Onnx</t>
@@ -1836,46 +1553,14 @@
           <t>베이스 모델</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1903,11 +1588,7 @@
           <t>https://huggingface.co/Supertone/supertonic-2</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>동일한 추론 속도를 유지하며 5개 언어로 확장된 66M 경량 온디바이스 TTS</t>
@@ -1933,29 +1614,17 @@
           <t>OpenRAIL</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-01-06</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2026-01-06</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
+      <c r="L3" s="2" t="n">
+        <v>46028</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>46028</v>
+      </c>
+      <c r="N3" s="3" t="n">
         <v>66000000</v>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
           <t>Onnx</t>
@@ -1971,41 +1640,13 @@
           <t>Supertone/supertonic</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2033,11 +1674,7 @@
           <t>https://huggingface.co/Supertone/supertonic-3</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>5개에서 31개 언어로 확장하고 낭독 안정성을 개선한 99M 파라미터 온디바이스 TTS</t>
@@ -2063,29 +1700,17 @@
           <t>OpenRAIL</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="N4" t="n">
+      <c r="L4" s="2" t="n">
+        <v>46148</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>46160</v>
+      </c>
+      <c r="N4" s="3" t="n">
         <v>99000000</v>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="O4" s="3" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
           <t>Onnx</t>
@@ -2096,46 +1721,14 @@
           <t>베이스 모델</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2193,20 +1786,16 @@
           <t>기타(hyperclovax)</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>2025-12-23</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2026-01-06</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
+      <c r="L5" s="2" t="n">
+        <v>46014</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>46028</v>
+      </c>
+      <c r="N5" s="3" t="n">
         <v>10741664520</v>
       </c>
-      <c r="O5" t="n">
+      <c r="O5" s="3" t="n">
         <v>32768</v>
       </c>
       <c r="P5" t="inlineStr">
@@ -2224,41 +1813,13 @@
           <t>베이스 모델</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr">
         <is>
           <t>2025-05</t>
@@ -2291,11 +1852,7 @@
           <t>https://huggingface.co/naver-hyperclovax/HyperCLOVAX-SEED-Text-Instruct-0.5B</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>동급 대비 수학·한국어 성능 우수, 학습비용 39배 절감돼 엣지 기기 배포에 적합한 소형 모델</t>
@@ -2321,20 +1878,16 @@
           <t>기타(hyperclovax-seed)</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>2025-04-22</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2025-07-21</t>
-        </is>
-      </c>
-      <c r="N6" t="n">
+      <c r="L6" s="2" t="n">
+        <v>45769</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>45859</v>
+      </c>
+      <c r="N6" s="3" t="n">
         <v>566281216</v>
       </c>
-      <c r="O6" t="n">
+      <c r="O6" s="3" t="n">
         <v>4096</v>
       </c>
       <c r="P6" t="inlineStr">
@@ -2362,31 +1915,15 @@
           <t>KMMLU=38.15;HAE-RAE=56.19;CLiCK=44.46;KoBEST=62.99</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr">
         <is>
           <t>KMMLU=38.15;HAE-RAE=56.19;CLiCK=44.46;KoBEST=62.99</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr">
         <is>
           <t>2025-01</t>
@@ -2449,20 +1986,16 @@
           <t>기타(hyperclovax-seed)</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>2025-07-21</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="N7" t="n">
+      <c r="L7" s="2" t="n">
+        <v>45859</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>46170</v>
+      </c>
+      <c r="N7" s="3" t="n">
         <v>14748112896</v>
       </c>
-      <c r="O7" t="n">
+      <c r="O7" s="3" t="n">
         <v>32768</v>
       </c>
       <c r="P7" t="inlineStr">
@@ -2480,11 +2013,7 @@
           <t>경량화·증류 모델</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
           <t>MMLU=71.21;BigBench-Hard=62.16;Hellaswag=61.25;Winogrande=75.93;PIQA=77.91;ARC-challenge=62.46;SocialIQa=52.05;MT-Bench=8.8313;Arena-Hard-v0.1=58.26;GPT4Eval=82.00;CLIcK=72.08;HAERAE-Bench=85.06;KOBEST=85.70;KorMedMCQA=64.11;KMMLU=54.28;KoBigBench=74.82;KoCommonGEN-v2=66.82;CSAT-ko-2025=75.16;KoBALT=45.00;LogicKor=8.74</t>
@@ -2495,31 +2024,15 @@
           <t>GSM8k=95.53;MATH500=93.80;HumanEval=94.51;MBPP=87.59</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr">
         <is>
           <t>CLIcK=72.08;HAERAE-Bench=85.06;KOBEST=85.70;KorMedMCQA=64.11;KMMLU=54.28;KoBigBench=74.82;KoCommonGEN-v2=66.82;CSAT-ko-2025=75.16;KoBALT=45.00;LogicKor=8.74</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2577,20 +2090,16 @@
           <t>기타(hyperclovax)</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>2025-12-23</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-07-14</t>
-        </is>
-      </c>
-      <c r="N8" t="n">
+      <c r="L8" s="2" t="n">
+        <v>46014</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>46217</v>
+      </c>
+      <c r="N8" s="3" t="n">
         <v>33313410304</v>
       </c>
-      <c r="O8" t="n">
+      <c r="O8" s="3" t="n">
         <v>131072</v>
       </c>
       <c r="P8" t="inlineStr">
@@ -2608,41 +2117,13 @@
           <t>베이스 모델</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr">
         <is>
           <t>2025-05</t>
@@ -2675,11 +2156,7 @@
           <t>https://huggingface.co/naver-hyperclovax/HyperCLOVAX-SEED-Vision-Instruct-3B</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>적은 비전 토큰으로도 한국어 VQA·이미지해석에서 동급 오픈소스 모델 대비 우수한 경량 VLM</t>
@@ -2705,20 +2182,16 @@
           <t>기타(hyperclovax-seed)</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>2025-04-22</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2025-09-16</t>
-        </is>
-      </c>
-      <c r="N9" t="n">
+      <c r="L9" s="2" t="n">
+        <v>45769</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>45916</v>
+      </c>
+      <c r="N9" s="3" t="n">
         <v>3721243520</v>
       </c>
-      <c r="O9" t="n">
+      <c r="O9" s="3" t="n">
         <v>16384</v>
       </c>
       <c r="P9" t="inlineStr">
@@ -2746,31 +2219,19 @@
           <t>KMMLU=44.22;HAE-RAE=64.99;CLiCK=55.99;KoBEST=71.80</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
           <t>VideoMME=48.2;NAVER-TV-CLIP=61.0;VideoChatGPT=53.6;PerceptionTest=55.2;ActivityNet-QA=50.6;KoNet=69.2;MMBench-Val=81.8;TextVQA-Val=79.2;Korean VisIT-Bench=37.0</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr">
         <is>
           <t>KMMLU=44.22;HAE-RAE=64.99;CLiCK=55.99;KoBEST=71.80;VideoMME=48.2;NAVER-TV-CLIP=61.0;VideoChatGPT=53.6;KoNet=69.2;Korean VisIT-Bench=37.0</t>
         </is>
       </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>미기재</t>
-        </is>
-      </c>
+      <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr">
         <is>
           <t>2024-08</t>

</xml_diff>